<commit_message>
Update Pinterest posting data
</commit_message>
<xml_diff>
--- a/data/amazon_products.xlsx
+++ b/data/amazon_products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -875,466 +875,6 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Trustous Men’s Pure Cotton Kurta Dhoti Set | Traditional Ethnic Wear for Festive, Wedding &amp; Puja Occasion</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/51a2QdCIA4L._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0H2FVJRHK?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Men’s Traditional Kurta for Men | Ethnic Wear Kurta for Festive, Wedding &amp; Casual Occasion | Stylish Regular Fit Kurta for Men</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/51KXtvGVB0L._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0H34STXNS?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Cotton Blend Self Design Printed Casual Short Kurta for Men Long Sleeve Mandarin Collar Stylish Kurta Shirt for Men</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/51n05rjWoiL._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0GK98CZPC?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>ROYALSCOUT Men's Cotton Polyester Blend Solid Regular Fit Full Sleeve Short Kurta | Ethnic, Lightweight Summer Kurta for Daily &amp; Occasion Use</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/61FWZ9dcQML._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0DHXFHNCH?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>LookMark Men’s Printed Silk Blend Kurta with Mandarin Collar, Full Sleeves, Straight Fit Traditional Ethnic Wear</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/51qygTxpJOL._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0GGC6H8YZ?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Zombom Cotton Polyester Blend Solid Casual Regular Fit Mandarin/Chinese Collor Short Kurta for Men</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/71nEy2iSx-L._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0D3XJHFJK?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Majestic Man Men's Cotton Regular Fit Casual Mandarin Collar Ethnic Motifs Printed Long Regular Kurta</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/711YfcFNl+L._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0CPWBVGLR?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>FINIVO FASHION Men’s Cotton Blend Short Kurta with Bold Printed Front Design | Full Sleeve Ethnic Casual Kurta with Mandarin Collar | Artistic Festival &amp; Travel Wear for Modern Ethnic Style</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/51XUrcCln+L._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0FJF7N7WD?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Trustous Men's Printed Kurta Dhoti Set Traditional Ethnic Wear for Festivals &amp; Weddings | Men's Stylish Printed Kurta with Dhoti Set | Traditional Indian Ethnic Wear for Men</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/41r5ITgctcL._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0H72RYHBY?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>DEELMO Men’s Cotton Blend Printed Long Sleeve Short Kurta | Stylish Casual &amp; Ethnic Wear | Comfortable Mandarin Collar Kurta for Daily, Festive &amp; Party Outfits</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/71vsX4HQH-L._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0FZJPMWRQ?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Men’s Lakhnawi Chikankari Cotton Blend Ethnic Wear Kurta for Men Knee Length Embroidered Kurta Mandarin Collar Full Sleeve Wedding Festive Party</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/71CMf5jpAFL._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0GXQ28WND?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Men’s Madhubani Printed Khadi Silk Kurta | Premium Ethnic Wear for Weddings &amp; Festivals | Traditional Art Design | Comfortable &amp; Stylish Outfit</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/41lfv5Bne2L._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0G448V51K?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Men Ethnic Gold Leaves 100% pure Jacquard Kurta &amp; Aladdin salwar special for Lohri &amp; New Year, In Panjabi Style</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/71MYoHK0krL._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0BS19ZN4K?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>ROYALSCOUT Men's Short Kurta | Solid Mandarin Collar Full Sleeve Pullover Style Kurta | Regular Fit Casual Ethnic Wear for Men</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/61xL-c8CR6L._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0CW1V697B?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>ROYALSCOUT Men's Cotton Polyester Blend Kurta Style Shirt with Mandarin Collar, Half Button Placket, Dual Chest Pockets, Long Sleeve Casual Ethnic Fusion Wear for Office, Festive and Daily Use</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/61BCD0tyMeL._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0GKVMSQWX?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Amazon Brand - Tavasya Men Printed Kurta with Ethnic Motif Border | Special Haldi Kurta | Festive Embellished Long Kurta | Embroidery Kurta | Ethnic Wear | Mandarin Collar | Knee Length</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/51MqzAFtWcL._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0GHYVS5SN?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Isha Life Organic Cotton Men Dhoti Pant | Elastic Waist Traditional Style Bottom Wear | Regular Fit Comfortable Casual &amp; Ethnic Wear for Men (S–XL)</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/61Ql4IqEenL._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0GMXXKV27?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Logass Kurta Pyjama Set for Mens Ethnic and Designer Wear Kurta Pyjama</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/51FE21IGnyS._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0BNJB7FZX?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>LATEST CHIKAN Men's Cotton Regular Textured Long Kurta Full Sleeves - Casual Ethnic Wear</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/611poKYvqQL._SY741_.jpg</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B08HK2ZRLP?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>DIVISIVE Men's Sequince Embroidered Cotton Blend Only Slim Fit Kurta</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/W/BW_MEDIAX_AVIF_MEASUREMENT_1306696-T1/images/I/71xULJlZzCL._SX679_.jpg</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>https://www.amazon.in/dp/B0CR9446X2?th=1&amp;psc=1</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>